<commit_message>
Project BugReproducing2-DEFAULT-2026-07-31_07-55-00 is saved.
</commit_message>
<xml_diff>
--- a/BugReproducing2-DEFAULT-2026-07-31_07-55-00/BugReproducing (1).xlsx
+++ b/BugReproducing2-DEFAULT-2026-07-31_07-55-00/BugReproducing (1).xlsx
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="19">
   <si>
     <t>a</t>
   </si>
@@ -93,6 +93,9 @@
   </si>
   <si>
     <t>5</t>
+  </si>
+  <si>
+    <t>3=</t>
   </si>
 </sst>
 </file>
@@ -468,7 +471,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{871B0360-4A65-8D4C-9F92-BAB28DCD4F5A}">
-  <dimension ref="B9:F17"/>
+  <dimension ref="B9:F18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="9" spans="2:6" x14ac:dyDescent="0.2">
@@ -494,15 +497,9 @@
       <c r="C11" s="0" t="s">
         <v>14</v>
       </c>
-      <c r="D11" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="E11" s="0" t="s">
-        <v>16</v>
-      </c>
-      <c r="F11" s="0" t="s">
-        <v>17</v>
-      </c>
+      <c r="D11" s="0"/>
+      <c r="E11" s="0"/>
+      <c r="F11" s="0"/>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B12" s="0" t="s">
@@ -516,37 +513,33 @@
       <c r="F12" s="1"/>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="0"/>
+      <c r="C13" s="0"/>
+      <c r="D13" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B14" s="0" t="s">
         <v>0</v>
       </c>
-      <c r="C13" s="0" t="n">
+      <c r="C14" s="0" t="n">
         <v>10.0</v>
       </c>
-      <c r="D13" s="0" t="n">
+      <c r="D14" s="0" t="n">
         <v>20.0</v>
       </c>
-      <c r="E13" s="0" t="n">
+      <c r="E14" s="0" t="n">
         <v>30.0</v>
       </c>
-      <c r="F13" s="0" t="n">
+      <c r="F14" s="0" t="n">
         <v>40.0</v>
-      </c>
-    </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B14" s="0" t="n">
-        <v>12.0</v>
-      </c>
-      <c r="C14" s="0" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="D14" s="0" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="E14" s="0" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="F14" s="0" t="n">
-        <v>0.0</v>
       </c>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.2">
@@ -597,6 +590,23 @@
         <v>0.0</v>
       </c>
       <c r="F17" t="n" s="0">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" t="n" s="0">
+        <v>12.0</v>
+      </c>
+      <c r="C18" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="D18" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="E18" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="F18" t="n" s="0">
         <v>0.0</v>
       </c>
     </row>

</xml_diff>